<commit_message>
video_eraser format test comit
</commit_message>
<xml_diff>
--- a/Log/Video_eraser_test_bug_log.xlsx
+++ b/Log/Video_eraser_test_bug_log.xlsx
@@ -4,12 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6900" activeTab="1"/>
+    <workbookView windowWidth="25280" windowHeight="11940" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="TestCase" sheetId="1" r:id="rId1"/>
-    <sheet name="Bug" sheetId="2" r:id="rId2"/>
-    <sheet name="bug_2.8.2_21_10" sheetId="3" r:id="rId3"/>
+    <sheet name="fomat_handle_test" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="126">
   <si>
     <t>TC</t>
   </si>
@@ -331,40 +330,98 @@
     <t>version: 2.8.2</t>
   </si>
   <si>
-    <t>Bug report ngày 16/10/2025</t>
+    <t>Step</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Ở màn review video trước khi vào màn hình edit chính, video đang được pause ở khoảng giữa</t>
-  </si>
-  <si>
-    <t>video không dừng từ khoảng 00:00 đến trước 00:01 hoặc ở khoảng cuối của video</t>
-  </si>
-  <si>
-    <t>Confirmed (accepted)</t>
-  </si>
-  <si>
-    <t>chức năng "force update"</t>
-  </si>
-  <si>
-    <t>Reject</t>
-  </si>
-  <si>
-    <t>Lỗi logic, giá trị skip_version &lt; lastest_version nhưng app vẫn bypass qua state "Optional update"; Đã được sửa vào ngày 22/10/2025 ở version 2.8.3 (Android)</t>
-  </si>
-  <si>
-    <t>closed</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>confirmed</t>
+    <t>Actual Output</t>
+  </si>
+  <si>
+    <t>FM01</t>
+  </si>
+  <si>
+    <t>sử dụng chức năng AI Filler, tài khoản hiện đang có 878</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File WEBM
+2. xử lý từ 00:00 đến 00:07
+3. tua video bằng thanh tiến trình
+4. lưu video về máy</t>
+  </si>
+  <si>
+    <t>Hiện lên màn processing, sau 1 khoảng thời gian, xuất hiện ra màn review video sau khi xử lý, video được lưu đúng với video trên project, tài khoản còn lại 858</t>
+  </si>
+  <si>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>chi phí xử lý 16</t>
+  </si>
+  <si>
+    <t>FM02</t>
+  </si>
+  <si>
+    <t>sử dụng chức năng AI Filler, tài khoản hiện đang có 110</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File MKV
+2. xử lý từ 00:00 đến 00:10
+3. tua video bằng thanh tiến trình
+4. lưu video về máy</t>
+  </si>
+  <si>
+    <t>Hiện lên màn processing, sau 2 khoảng thời gian, xuất hiện ra màn review video sau khi xử lý, video được lưu đúng với video trên project, tài khoản còn lại 90</t>
+  </si>
+  <si>
+    <t>chi phí xử lý 20</t>
+  </si>
+  <si>
+    <t>FM03</t>
+  </si>
+  <si>
+    <t>sử dụng chức năng AI Filler, tài khoản hiện đang có 90</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File MP4(h264)
+2. xử lý từ 00:00 đến 00:10
+3. tua video bằng thanh tiến trình
+4. lưu video về máy</t>
+  </si>
+  <si>
+    <t>Hiện lên màn processing, sau 3 khoảng thời gian, xuất hiện ra màn review video sau khi xử lý, video được lưu đúng với video trên project, tài khoản còn lại 70</t>
+  </si>
+  <si>
+    <t>FM04</t>
+  </si>
+  <si>
+    <t>sử dụng chức năng AI Filler, tài khoản hiện đang có 70</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File MP4(AV1)
+2. xử lý từ 00:00 đến 00:10
+3. Chọn button xem sau
+4. Thoát ra khỏi app
+5. Nhấn vào thông báo xử lý xong 
+6. Nhấn vào project
+6. tua video bằng thanh tiến trình
+7. lưu video về máy</t>
+  </si>
+  <si>
+    <t>trình tự xuất hiện từ màn chọn video đến màn processing giống các TC từFM01 đến FM03, Sau khi nhấn thông báo vào thẳng đến màn review sau khi xử lý, video được lưu đúng với trên project, tài khoản còn lại 50</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>chi phí xử lý 20, Lỗi không thể xử lý định dạng file AV1</t>
+  </si>
+  <si>
+    <t>Trình tự xuất hiện từ màn chọn video đến màn processing giống các TC từ FM01 đến FM03, nhấn thông báo vào màn app, vào màn review project, vid không hiện, thanh tiến trình video treo, không thể tua</t>
+  </si>
+  <si>
+    <t>3 TC FM01, 02, 03 được khắc phục ở bản 2.8.7</t>
   </si>
 </sst>
 </file>
@@ -378,7 +435,7 @@
     <numFmt numFmtId="179" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
     <numFmt numFmtId="180" formatCode="h:mm\ AM/PM"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -389,14 +446,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -902,143 +951,161 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1051,53 +1118,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="58" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="58" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1633,679 +1673,679 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="8.8828125" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="4.33333333333333" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.8857142857143" style="3" customWidth="1"/>
-    <col min="3" max="3" width="21.1428571428571" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.8571428571429" style="4" customWidth="1"/>
-    <col min="5" max="5" width="26.5714285714286" style="4" customWidth="1"/>
-    <col min="6" max="6" width="29.1142857142857" style="4" customWidth="1"/>
-    <col min="7" max="7" width="22.3333333333333" style="4" customWidth="1"/>
-    <col min="8" max="8" width="11.447619047619" style="7"/>
-    <col min="9" max="9" width="23.8571428571429" style="7" customWidth="1"/>
-    <col min="10" max="16384" width="8.88571428571429" style="7"/>
+    <col min="1" max="1" width="4.3359375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="33.8828125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="25.859375" style="10" customWidth="1"/>
+    <col min="5" max="5" width="26.5703125" style="10" customWidth="1"/>
+    <col min="6" max="6" width="29.1171875" style="10" customWidth="1"/>
+    <col min="7" max="7" width="22.3359375" style="10" customWidth="1"/>
+    <col min="8" max="8" width="11.4453125" style="11"/>
+    <col min="9" max="9" width="23.859375" style="11" customWidth="1"/>
+    <col min="10" max="16384" width="8.8828125" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" s="13" customFormat="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="4" customFormat="1" ht="17" spans="1:7">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" s="13" customFormat="1" spans="1:7">
-      <c r="A2" s="16">
+    <row r="2" s="4" customFormat="1" spans="1:7">
+      <c r="A2" s="12">
         <v>45946</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-    </row>
-    <row r="3" s="14" customFormat="1" ht="30" spans="1:7">
-      <c r="A3" s="2">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" s="5" customFormat="1" ht="34" spans="1:7">
+      <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="4"/>
-    </row>
-    <row r="4" s="15" customFormat="1" ht="43" customHeight="1" spans="1:7">
-      <c r="A4" s="2">
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" s="6" customFormat="1" ht="43" customHeight="1" spans="1:7">
+      <c r="A4" s="8">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="4"/>
-    </row>
-    <row r="5" s="15" customFormat="1" ht="30" spans="1:7">
-      <c r="A5" s="2">
+      <c r="G4" s="10"/>
+    </row>
+    <row r="5" s="6" customFormat="1" ht="17" spans="1:7">
+      <c r="A5" s="8">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" s="6" customFormat="1" spans="1:7">
-      <c r="A6" s="2">
+      <c r="G5" s="10"/>
+    </row>
+    <row r="6" s="7" customFormat="1" ht="17" spans="1:7">
+      <c r="A6" s="8">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" customFormat="1" customHeight="1" spans="1:8">
-      <c r="A7" s="2">
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" customFormat="1" ht="15" customHeight="1" spans="1:8">
+      <c r="A7" s="8">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="17"/>
     </row>
     <row r="8" ht="31" customHeight="1" spans="1:8">
-      <c r="A8" s="2">
+      <c r="A8" s="8">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="17"/>
     </row>
     <row r="9" ht="33" customHeight="1" spans="1:8">
-      <c r="A9" s="2">
+      <c r="A9" s="8">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H9" s="19"/>
-    </row>
-    <row r="10" ht="45" spans="1:8">
-      <c r="A10" s="2">
+      <c r="H9" s="18"/>
+    </row>
+    <row r="10" ht="34" spans="1:8">
+      <c r="A10" s="8">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="19"/>
-    </row>
-    <row r="11" ht="45" spans="1:8">
-      <c r="A11" s="2">
+      <c r="H10" s="18"/>
+    </row>
+    <row r="11" ht="34" spans="1:8">
+      <c r="A11" s="8">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="19"/>
+      <c r="H11" s="18"/>
     </row>
     <row r="12" ht="77" customHeight="1" spans="1:8">
-      <c r="A12" s="2">
+      <c r="A12" s="8">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="19"/>
-    </row>
-    <row r="13" ht="45" spans="1:8">
-      <c r="A13" s="2">
+      <c r="H12" s="18"/>
+    </row>
+    <row r="13" ht="34" spans="1:8">
+      <c r="A13" s="8">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="H13" s="19"/>
-    </row>
-    <row r="14" ht="45" spans="1:8">
-      <c r="A14" s="2">
+      <c r="H13" s="18"/>
+    </row>
+    <row r="14" ht="51" spans="1:8">
+      <c r="A14" s="8">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H14" s="19"/>
+      <c r="H14" s="18"/>
     </row>
     <row r="15" spans="8:8">
-      <c r="H15" s="19"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="19"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="18"/>
     </row>
     <row r="17" ht="81" customHeight="1" spans="1:8">
-      <c r="A17" s="2">
+      <c r="A17" s="8">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="H17" s="19"/>
-    </row>
-    <row r="18" ht="120" spans="1:8">
-      <c r="A18" s="2">
+      <c r="H17" s="18"/>
+    </row>
+    <row r="18" ht="118" spans="1:8">
+      <c r="A18" s="8">
         <v>14</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="H18" s="19"/>
-    </row>
-    <row r="19" ht="150" spans="1:8">
-      <c r="A19" s="2">
+      <c r="H18" s="18"/>
+    </row>
+    <row r="19" ht="152" spans="1:8">
+      <c r="A19" s="8">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="H19" s="19"/>
-    </row>
-    <row r="20" ht="150" spans="1:8">
-      <c r="A20" s="2">
+      <c r="H19" s="18"/>
+    </row>
+    <row r="20" ht="152" spans="1:8">
+      <c r="A20" s="8">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="19"/>
-    </row>
-    <row r="21" ht="90" spans="1:8">
-      <c r="A21" s="2">
+      <c r="H20" s="18"/>
+    </row>
+    <row r="21" ht="101" spans="1:8">
+      <c r="A21" s="8">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H21" s="19"/>
-    </row>
-    <row r="22" ht="45" spans="1:8">
-      <c r="A22" s="2">
+      <c r="H21" s="18"/>
+    </row>
+    <row r="22" ht="34" spans="1:8">
+      <c r="A22" s="8">
         <v>18</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="H22" s="19"/>
-    </row>
-    <row r="23" ht="60" spans="1:8">
-      <c r="A23" s="2">
+      <c r="H22" s="18"/>
+    </row>
+    <row r="23" ht="68" spans="1:8">
+      <c r="A23" s="8">
         <v>19</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="H23" s="19"/>
-    </row>
-    <row r="24" ht="60" spans="1:8">
-      <c r="A24" s="2">
+      <c r="H23" s="18"/>
+    </row>
+    <row r="24" ht="68" spans="1:8">
+      <c r="A24" s="8">
         <v>20</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="H24" s="19"/>
-    </row>
-    <row r="25" ht="45" spans="1:8">
-      <c r="A25" s="2">
+      <c r="H24" s="18"/>
+    </row>
+    <row r="25" ht="34" spans="1:8">
+      <c r="A25" s="8">
         <v>21</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H25" s="19"/>
-    </row>
-    <row r="26" ht="30" spans="1:8">
-      <c r="A26" s="2">
+      <c r="H25" s="18"/>
+    </row>
+    <row r="26" ht="34" spans="1:8">
+      <c r="A26" s="8">
         <v>22</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="H26" s="19"/>
-    </row>
-    <row r="27" ht="45" spans="1:8">
-      <c r="A27" s="2">
+      <c r="H26" s="18"/>
+    </row>
+    <row r="27" ht="51" spans="1:8">
+      <c r="A27" s="8">
         <v>23</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="H27" s="19"/>
-    </row>
-    <row r="28" ht="60" spans="1:8">
-      <c r="A28" s="2">
+      <c r="H27" s="18"/>
+    </row>
+    <row r="28" ht="68" spans="1:8">
+      <c r="A28" s="8">
         <v>24</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="H28" s="19"/>
+      <c r="H28" s="18"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="19"/>
-    </row>
-    <row r="30" ht="75" spans="1:7">
-      <c r="A30" s="2">
+      <c r="B29" s="16"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="18"/>
+    </row>
+    <row r="30" ht="84" spans="1:7">
+      <c r="A30" s="8">
         <v>25</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="31" ht="120" spans="1:7">
-      <c r="A31" s="2">
+    <row r="31" ht="118" spans="1:7">
+      <c r="A31" s="8">
         <v>26</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="32" ht="150" spans="1:7">
-      <c r="A32" s="2">
+    <row r="32" ht="135" spans="1:7">
+      <c r="A32" s="8">
         <v>27</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="10" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2324,266 +2364,136 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="29.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="25.7809523809524" customWidth="1"/>
-    <col min="4" max="4" width="19.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="20.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="25.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="11.8571428571429" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="1" max="1" width="5.46875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.0078125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.4765625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="27.078125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.8515625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.8359375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.25" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" spans="1:7">
-      <c r="A1" s="8" t="s">
+    <row r="1" ht="17" spans="1:7">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-    </row>
-    <row r="6" s="6" customFormat="1" spans="1:9">
-      <c r="A6" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="E1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="I6" s="6" t="s">
+      <c r="G1" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="7" s="7" customFormat="1" ht="57" customHeight="1" spans="1:9">
-      <c r="A7" s="9">
-        <v>10</v>
-      </c>
-      <c r="B7" s="7" t="s">
+    <row r="2" ht="125" customHeight="1" spans="1:6">
+      <c r="A2" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="C2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I7" s="11">
-        <v>45946</v>
-      </c>
-    </row>
-    <row r="8" customFormat="1" spans="1:9">
-      <c r="A8" s="10" t="s">
+      <c r="D2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-    </row>
-    <row r="9" ht="105" spans="1:9">
-      <c r="A9" s="2">
-        <v>26</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="E2" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="I9" s="12">
-        <v>45951.4513888889</v>
-      </c>
-    </row>
-    <row r="10" ht="90" spans="1:9">
-      <c r="A10" s="5">
-        <v>25</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="F2" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="H10" t="s">
+    </row>
+    <row r="3" ht="101" spans="1:6">
+      <c r="A3" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="I10" s="12">
-        <v>45952</v>
-      </c>
+      <c r="B3" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" ht="118" spans="1:6">
+      <c r="A4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" ht="202" spans="1:7">
+      <c r="A5" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="4:6">
+      <c r="D7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A8:I8"/>
+  <mergeCells count="1">
+    <mergeCell ref="D7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="7"/>
-  <cols>
-    <col min="1" max="1" width="4.14285714285714" customWidth="1"/>
-    <col min="2" max="2" width="33.4285714285714" customWidth="1"/>
-    <col min="3" max="3" width="18.1428571428571" customWidth="1"/>
-    <col min="4" max="4" width="22.2857142857143" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="24.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="29.2857142857143" customWidth="1"/>
-    <col min="8" max="8" width="10.4285714285714" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" ht="105" customHeight="1" spans="1:8">
-      <c r="A2" s="2">
-        <v>26</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="H2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" ht="60" spans="1:8">
-      <c r="A3" s="5">
-        <v>25</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="H3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Force upade ME commit
</commit_message>
<xml_diff>
--- a/Log/Video_eraser_test_bug_log.xlsx
+++ b/Log/Video_eraser_test_bug_log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25280" windowHeight="11940" activeTab="1"/>
+    <workbookView windowWidth="18700" windowHeight="16340" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="TestCase" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="137">
   <si>
     <t>TC</t>
   </si>
@@ -337,6 +337,9 @@
   </si>
   <si>
     <t>Actual Output</t>
+  </si>
+  <si>
+    <t>Android</t>
   </si>
   <si>
     <t>FM01</t>
@@ -421,7 +424,49 @@
     <t>Trình tự xuất hiện từ màn chọn video đến màn processing giống các TC từ FM01 đến FM03, nhấn thông báo vào màn app, vào màn review project, vid không hiện, thanh tiến trình video treo, không thể tua</t>
   </si>
   <si>
-    <t>3 TC FM01, 02, 03 được khắc phục ở bản 2.8.7</t>
+    <t>IOS</t>
+  </si>
+  <si>
+    <t>FM05</t>
+  </si>
+  <si>
+    <t>Sử dụng chức năng AI Filter, tài khoản đang có trên 20 credits</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File 3GP
+2. xử lý từ 00:00 đến 00:10
+3. tua video bằng thanh tiến trình
+4. lưu video về máy</t>
+  </si>
+  <si>
+    <t>Hiện lên màn processing, sau 3 khoảng thời gian, xuất hiện ra màn review video sau khi xử lý, thao tác tua trên thanh duration được phản hồi đúng, video được lưu đúng với video trên project, tài khoản bị trừ đi 20 credits</t>
+  </si>
+  <si>
+    <t>FM06</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File 3G2
+2. xử lý từ 00:00 đến 00:10
+3. tua video bằng thanh tiến trình
+5. lưu video về máy</t>
+  </si>
+  <si>
+    <t>FM07</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File MOV
+2. xử lý từ 00:00 đến 00:10
+3. tua video bằng thanh tiến trình
+6. lưu video về máy</t>
+  </si>
+  <si>
+    <t>FM08</t>
+  </si>
+  <si>
+    <t>1. chọn xử lý File MP4
+2. xử lý từ 00:00 đến 00:10
+3. tua video bằng thanh tiến trình
+6. lưu video về máy</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1126,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1094,6 +1139,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1113,9 +1164,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="58" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1675,19 +1723,19 @@
   <dimension ref="A1:H32"/>
   <sheetFormatPr defaultColWidth="8.8828125" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="4.3359375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="33.8828125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="25.859375" style="10" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" style="10" customWidth="1"/>
-    <col min="6" max="6" width="29.1171875" style="10" customWidth="1"/>
-    <col min="7" max="7" width="22.3359375" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.4453125" style="11"/>
-    <col min="9" max="9" width="23.859375" style="11" customWidth="1"/>
-    <col min="10" max="16384" width="8.8828125" style="11"/>
+    <col min="1" max="1" width="4.3359375" style="10" customWidth="1"/>
+    <col min="2" max="2" width="33.8828125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="12" customWidth="1"/>
+    <col min="4" max="4" width="25.859375" style="12" customWidth="1"/>
+    <col min="5" max="5" width="26.5703125" style="12" customWidth="1"/>
+    <col min="6" max="6" width="29.1171875" style="12" customWidth="1"/>
+    <col min="7" max="7" width="22.3359375" style="12" customWidth="1"/>
+    <col min="8" max="8" width="11.4453125" style="1"/>
+    <col min="9" max="9" width="23.859375" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.8828125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="1" ht="17" spans="1:7">
+    <row r="1" s="6" customFormat="1" ht="17" spans="1:7">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1710,642 +1758,642 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" s="4" customFormat="1" spans="1:7">
-      <c r="A2" s="12">
+    <row r="2" s="6" customFormat="1" spans="1:7">
+      <c r="A2" s="13">
         <v>45946</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-    </row>
-    <row r="3" s="5" customFormat="1" ht="34" spans="1:7">
-      <c r="A3" s="8">
+      <c r="B2" s="14"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+    </row>
+    <row r="3" s="7" customFormat="1" ht="34" spans="1:7">
+      <c r="A3" s="10">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="10"/>
-    </row>
-    <row r="4" s="6" customFormat="1" ht="43" customHeight="1" spans="1:7">
-      <c r="A4" s="8">
+      <c r="G3" s="12"/>
+    </row>
+    <row r="4" s="8" customFormat="1" ht="43" customHeight="1" spans="1:7">
+      <c r="A4" s="10">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="10"/>
-    </row>
-    <row r="5" s="6" customFormat="1" ht="17" spans="1:7">
-      <c r="A5" s="8">
+      <c r="G4" s="12"/>
+    </row>
+    <row r="5" s="8" customFormat="1" ht="17" spans="1:7">
+      <c r="A5" s="10">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="10"/>
-    </row>
-    <row r="6" s="7" customFormat="1" ht="17" spans="1:7">
-      <c r="A6" s="8">
+      <c r="G5" s="12"/>
+    </row>
+    <row r="6" s="9" customFormat="1" ht="17" spans="1:7">
+      <c r="A6" s="10">
         <v>4</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="10"/>
+      <c r="G6" s="12"/>
     </row>
     <row r="7" customFormat="1" ht="15" customHeight="1" spans="1:8">
-      <c r="A7" s="8">
+      <c r="A7" s="10">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="10"/>
-      <c r="H7" s="17"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="18"/>
     </row>
     <row r="8" ht="31" customHeight="1" spans="1:8">
-      <c r="A8" s="8">
+      <c r="A8" s="10">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="17"/>
+      <c r="H8" s="18"/>
     </row>
     <row r="9" ht="33" customHeight="1" spans="1:8">
-      <c r="A9" s="8">
+      <c r="A9" s="10">
         <v>7</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H9" s="18"/>
+      <c r="H9" s="19"/>
     </row>
     <row r="10" ht="34" spans="1:8">
-      <c r="A10" s="8">
+      <c r="A10" s="10">
         <v>8</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="18"/>
+      <c r="H10" s="19"/>
     </row>
     <row r="11" ht="34" spans="1:8">
-      <c r="A11" s="8">
+      <c r="A11" s="10">
         <v>9</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="18"/>
+      <c r="H11" s="19"/>
     </row>
     <row r="12" ht="77" customHeight="1" spans="1:8">
-      <c r="A12" s="8">
+      <c r="A12" s="10">
         <v>10</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="18"/>
+      <c r="H12" s="19"/>
     </row>
     <row r="13" ht="34" spans="1:8">
-      <c r="A13" s="8">
+      <c r="A13" s="10">
         <v>11</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="H13" s="18"/>
+      <c r="H13" s="19"/>
     </row>
     <row r="14" ht="51" spans="1:8">
-      <c r="A14" s="8">
+      <c r="A14" s="10">
         <v>12</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H14" s="18"/>
+      <c r="H14" s="19"/>
     </row>
     <row r="15" spans="8:8">
-      <c r="H15" s="18"/>
+      <c r="H15" s="19"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="18"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="19"/>
     </row>
     <row r="17" ht="81" customHeight="1" spans="1:8">
-      <c r="A17" s="8">
+      <c r="A17" s="10">
         <v>13</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="H17" s="18"/>
+      <c r="H17" s="19"/>
     </row>
     <row r="18" ht="118" spans="1:8">
-      <c r="A18" s="8">
+      <c r="A18" s="10">
         <v>14</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="H18" s="18"/>
+      <c r="H18" s="19"/>
     </row>
     <row r="19" ht="152" spans="1:8">
-      <c r="A19" s="8">
+      <c r="A19" s="10">
         <v>15</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="H19" s="18"/>
+      <c r="H19" s="19"/>
     </row>
     <row r="20" ht="152" spans="1:8">
-      <c r="A20" s="8">
+      <c r="A20" s="10">
         <v>16</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="18"/>
+      <c r="H20" s="19"/>
     </row>
     <row r="21" ht="101" spans="1:8">
-      <c r="A21" s="8">
+      <c r="A21" s="10">
         <v>17</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="H21" s="18"/>
+      <c r="H21" s="19"/>
     </row>
     <row r="22" ht="34" spans="1:8">
-      <c r="A22" s="8">
+      <c r="A22" s="10">
         <v>18</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="H22" s="18"/>
+      <c r="H22" s="19"/>
     </row>
     <row r="23" ht="68" spans="1:8">
-      <c r="A23" s="8">
+      <c r="A23" s="10">
         <v>19</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="H23" s="18"/>
+      <c r="H23" s="19"/>
     </row>
     <row r="24" ht="68" spans="1:8">
-      <c r="A24" s="8">
+      <c r="A24" s="10">
         <v>20</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="H24" s="18"/>
+      <c r="H24" s="19"/>
     </row>
     <row r="25" ht="34" spans="1:8">
-      <c r="A25" s="8">
+      <c r="A25" s="10">
         <v>21</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="G25" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="H25" s="18"/>
+      <c r="H25" s="19"/>
     </row>
     <row r="26" ht="34" spans="1:8">
-      <c r="A26" s="8">
+      <c r="A26" s="10">
         <v>22</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="H26" s="18"/>
+      <c r="H26" s="19"/>
     </row>
     <row r="27" ht="51" spans="1:8">
-      <c r="A27" s="8">
+      <c r="A27" s="10">
         <v>23</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="G27" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="H27" s="18"/>
+      <c r="H27" s="19"/>
     </row>
     <row r="28" ht="68" spans="1:8">
-      <c r="A28" s="8">
+      <c r="A28" s="10">
         <v>24</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="H28" s="18"/>
+      <c r="H28" s="19"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="18"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="19"/>
     </row>
     <row r="30" ht="84" spans="1:7">
-      <c r="A30" s="8">
+      <c r="A30" s="10">
         <v>25</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" s="12" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="31" ht="118" spans="1:7">
-      <c r="A31" s="8">
+      <c r="A31" s="10">
         <v>26</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="G31" s="12" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="32" ht="135" spans="1:7">
-      <c r="A32" s="8">
+      <c r="A32" s="10">
         <v>27</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="F32" s="10" t="s">
+      <c r="F32" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="G32" s="12" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2364,8 +2412,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="6"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="5.46875" style="1" customWidth="1"/>
     <col min="2" max="2" width="19.0078125" style="1" customWidth="1"/>
@@ -2400,98 +2448,197 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" ht="125" customHeight="1" spans="1:6">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7">
+      <c r="A2" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" ht="125" customHeight="1" spans="1:6">
+      <c r="A3" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="3" ht="101" spans="1:6">
-      <c r="A3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="1" t="s">
+    </row>
+    <row r="4" ht="101" spans="1:6">
+      <c r="A4" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="4" ht="118" spans="1:6">
-      <c r="A4" s="1" t="s">
+      <c r="E4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="5" ht="118" spans="1:6">
+      <c r="A5" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" ht="202" spans="1:7">
-      <c r="A5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="E5" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" ht="202" spans="1:7">
+      <c r="A6" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="7" spans="4:6">
-      <c r="D7" s="2" t="s">
+      <c r="G6" s="1" t="s">
         <v>125</v>
       </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
       <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" ht="135" spans="1:7">
+      <c r="A8" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" ht="135" spans="1:7">
+      <c r="A9" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" ht="135" spans="1:6">
+      <c r="A10" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" ht="135" spans="1:6">
+      <c r="A11" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>114</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D7:F7"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A7:G7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>